<commit_message>
chore: organize theory files and update gitignore
</commit_message>
<xml_diff>
--- a/numpy/py_note.xlsx
+++ b/numpy/py_note.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22175" windowHeight="9720"/>
+    <workbookView windowWidth="22188" windowHeight="9720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>STT</t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>Ghi chú</t>
-  </si>
-  <si>
-    <t>Test python, in là print</t>
   </si>
   <si>
     <t>Tên</t>
@@ -1456,9 +1453,7 @@
         <f>IF(B2="","",SUM($E$2:E2)/TIME([1]Settings!$B$2,0,0))</f>
         <v/>
       </c>
-      <c r="I2" s="11" t="s">
-        <v>9</v>
-      </c>
+      <c r="I2" s="11"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10">
@@ -3775,7 +3770,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{bcbdea7a-cbbf-4c35-8468-7cb75a0ce538}</x14:id>
+          <x14:id>{5ff0c6ce-b325-415d-aeb6-264d665896e7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3794,7 +3789,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{bcbdea7a-cbbf-4c35-8468-7cb75a0ce538}">
+          <x14:cfRule type="dataBar" id="{5ff0c6ce-b325-415d-aeb6-264d665896e7}">
             <x14:dataBar minLength="10" maxLength="90" negativeBarColorSameAsPositive="1">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -3821,15 +3816,15 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
       <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3">
         <v>1</v>
@@ -3837,15 +3832,15 @@
     </row>
     <row r="3" s="1" customFormat="1" spans="1:2">
       <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3">
         <v>1</v>
@@ -3853,7 +3848,7 @@
     </row>
     <row r="5" s="1" customFormat="1" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1">
         <v>5</v>
@@ -3861,10 +3856,10 @@
     </row>
     <row r="6" s="1" customFormat="1" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" spans="1:2">
@@ -3872,7 +3867,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>